<commit_message>
Reword CVE acronym to plain language across proposal and workbook
Replace 'zero CVEs' phrasing with 'zero publicly registered security
vulnerabilities' to avoid confusion with CVs (curricula vitae) while
preserving the zero-breach / zero-vulnerability differentiator claim

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ypYFL7E2g6EXFAxcDeuoe
</commit_message>
<xml_diff>
--- a/PUCSL_Submission_Response_Workbook.xlsx
+++ b/PUCSL_Submission_Response_Workbook.xlsx
@@ -338,7 +338,7 @@
     <t>Abatis/Platinum company profile &amp; credentials pack</t>
   </si>
   <si>
-    <t>20+ yrs CNI protection; first client Swiss government/military; zero reported breaches, zero CVEs; deployments incl. Gulf smart-city OT programmes</t>
+    <t>20+ yrs CNI protection; first client Swiss government/military; zero reported breaches, zero registered vulnerabilities; deployments incl. Gulf smart-city OT programmes</t>
   </si>
   <si>
     <t>Platinum/Abatis financial statements (if required of both JV partners)</t>
@@ -1070,7 +1070,7 @@
     <t>Technical partner track record?</t>
   </si>
   <si>
-    <t>Abatis: Swiss company incorporated Oct 2004; first client was the Swiss government — technology designed at the request of the Swiss government and implemented by the Swiss military for CNI protection. In 20+ years: zero reported breaches against the code and zero CVEs registered — both believed unique in the industry.</t>
+    <t>Abatis: Swiss company incorporated Oct 2004; first client was the Swiss government — technology designed at the request of the Swiss government and implemented by the Swiss military for CNI protection. In 20+ years: zero reported breaches against the code and zero publicly registered security vulnerabilities — both believed unique in the industry.</t>
   </si>
   <si>
     <t>What differentiates the technical approach?</t>

</xml_diff>